<commit_message>
V1.3.4 Fixed BotReload not working Use new settings tabs to configure keys
</commit_message>
<xml_diff>
--- a/Chinese.xlsx
+++ b/Chinese.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SteamLibrary\steamapps\common\Barotrauma\LocalMods\Vanilla Components Expanded\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85F11B65-498A-4F9B-90A7-BF1FF216D0AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F2D7860-FDE7-4BDF-A31F-49E195399982}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="61">
   <si>
     <t>字段名</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -263,6 +263,10 @@
   </si>
   <si>
     <t>Lerp(reload, reload*4, 1-reload)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>已弃用</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -286,13 +290,19 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="12">
     <border>
@@ -425,7 +435,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -461,6 +471,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -857,23 +873,25 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="11"/>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5" t="s">
+      <c r="E5" s="13"/>
+      <c r="F5" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="H5" s="4"/>
+      <c r="H5" s="4" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
@@ -923,25 +941,27 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="10"/>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="D8" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="E8" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="F8" s="1" t="s">
+      <c r="E8" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="F8" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="G8" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="H8" s="4"/>
+      <c r="H8" s="4" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="10"/>

</xml_diff>